<commit_message>
Articulos - Edu Com - perfil
</commit_message>
<xml_diff>
--- a/data/edu_comp_en.xlsx
+++ b/data/edu_comp_en.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\Mile_CV\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Documents\GitHub\Mile_CV\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DBAA3B9-1EF2-4EC0-9F87-E78B9C7FE092}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{560EA78D-ACBE-4C27-9254-1BACBCE69A05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1815" yWindow="1815" windowWidth="21600" windowHeight="11505" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="education" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="0"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="11">
   <si>
     <t>what</t>
   </si>
@@ -45,9 +45,6 @@
     <t>Diploma in University Teaching</t>
   </si>
   <si>
-    <t>Diplomado en Diseño y Uso Pedagógico de Ambientes Virtuales de Aprendizaje Mediados por las TIC y las TAC</t>
-  </si>
-  <si>
     <t xml:space="preserve">Bogotá, Colombia </t>
   </si>
   <si>
@@ -55,6 +52,12 @@
   </si>
   <si>
     <t>Universidad El Bosque</t>
+  </si>
+  <si>
+    <t>Professional Certificate in Instructional Design and Virtual Learning Environments</t>
+  </si>
+  <si>
+    <t>Specialization in Teaching in Higher Education</t>
   </si>
 </sst>
 </file>
@@ -110,7 +113,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
     <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
@@ -406,17 +409,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E3"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="35.28515625" customWidth="1"/>
-    <col min="2" max="2" width="19.28515625" customWidth="1"/>
-    <col min="3" max="3" width="29.7109375" customWidth="1"/>
-    <col min="4" max="4" width="21.28515625" customWidth="1"/>
-    <col min="5" max="5" width="135.7109375" customWidth="1"/>
+    <col min="1" max="1" width="67" customWidth="1"/>
+    <col min="2" max="2" width="19.33203125" customWidth="1"/>
+    <col min="3" max="3" width="29.6640625" customWidth="1"/>
+    <col min="4" max="4" width="21.33203125" customWidth="1"/>
+    <col min="5" max="5" width="135.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -433,32 +436,46 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2">
+        <v>2026</v>
+      </c>
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" t="s">
         <v>6</v>
       </c>
-      <c r="B2">
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3">
         <v>2020</v>
-      </c>
-      <c r="C2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3">
-        <v>2019</v>
       </c>
       <c r="C3" t="s">
         <v>8</v>
       </c>
       <c r="D3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4">
+        <v>2019</v>
+      </c>
+      <c r="C4" t="s">
         <v>7</v>
+      </c>
+      <c r="D4" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>